<commit_message>
feat(catalog): render per-level sources and why lines
</commit_message>
<xml_diff>
--- a/data/capabilities.xlsx
+++ b/data/capabilities.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Proficiency Scale" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Scope Levels" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Domains" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sources &amp; Theory" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32267,4 +32268,256 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Citation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>dreyfus1980</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>theory</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Dreyfus &amp; Dreyfus, A Five-Stage Model of the Mental Activities Involved in Directed Skill Acquisition (1980)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.dtic.mil/sti/citations/ADA084551</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Basis of the P1-P6 proficiency bands</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>tuckman1965</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>theory</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Tuckman, Developmental Sequence in Small Groups, Psychological Bulletin 63(6), 384-399 (1965)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1037/h0022100</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Forming-storming-norming-performing team stages</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>bauer2010</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>empirical</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Bauer, Onboarding New Employees: Maximizing Success, SHRM Foundation Effective Practice Guidelines (2010)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shrm.org/content/dam/en/shrm/topics-tools/news/talent-acquisition/Onboarding-New-Employees.pdf</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Structured onboarding levels and outcomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>watkins2003</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>theory</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Watkins, The First 90 Days (Harvard Business Review Press, 2003)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>30/60/90 transition and ramp planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>sfia9</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>SFIA Foundation, Skills Framework for the Information Age, version 9 (2024)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://sfia-online.org/en/sfia-9</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Seven-level responsibility descriptors used as leveling standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>gitlab-em-jd</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>company-ladder</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>GitLab Handbook, Engineering Management Job Framework (accessed 2026-07)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://handbook.gitlab.com/job-families/engineering/engineering-management/</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Published EM/Senior EM/Director requirement deltas</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>skelton-pais2019</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>theory</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Team boundaries; org-level team formation patterns</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>haspeslagh1991</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>theory</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Haspeslagh &amp; Jemison, Managing Acquisitions: Creating Value Through Corporate Renewal (Free Press, 1991)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Integration design for step-change organizational growth</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>